<commit_message>
test(sparklines): measure same-day order — by time, not by cell (date-fractional row 5)
Review finding: rows 1 and 3 could not tell time order from cell order. Row 5
puts day-45000 times in reverse cell order; Excel leaves the day from the
latest time, so the full-serial sort is confirmed and pinned in the resolve
test. Doc: floored (not truncated), negative and near-midnight serials
unmeasured; date-fractional tolerance refit (0.005 / 0.029 / 71).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016KTccUzeFqqMqTthqgFm9H
</commit_message>
<xml_diff>
--- a/tests/fixtures/xlsx-sparklines/date-fractional-bordered.xlsx
+++ b/tests/fixtures/xlsx-sparklines/date-fractional-bordered.xlsx
@@ -280,7 +280,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="10" max="10" width="40.7109375" customWidth="1"/>
@@ -394,6 +394,33 @@
       </c>
       <c r="J4" s="1"/>
     </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>7</v>
+      </c>
+      <c r="C5">
+        <v>3</v>
+      </c>
+      <c r="D5">
+        <v>9</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>8</v>
+      </c>
+      <c r="G5">
+        <v>5</v>
+      </c>
+      <c r="H5">
+        <v>6</v>
+      </c>
+      <c r="J5" s="1"/>
+    </row>
     <row r="7">
       <c r="A7">
         <v>45000</v>
@@ -470,6 +497,32 @@
       </c>
       <c r="H9">
         <v>45030.5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>45000.5</v>
+      </c>
+      <c r="B10">
+        <v>45000.25</v>
+      </c>
+      <c r="C10">
+        <v>45000</v>
+      </c>
+      <c r="D10">
+        <v>45001</v>
+      </c>
+      <c r="E10">
+        <v>45002</v>
+      </c>
+      <c r="F10">
+        <v>45003</v>
+      </c>
+      <c r="G10">
+        <v>45004</v>
+      </c>
+      <c r="H10">
+        <v>45005</v>
       </c>
     </row>
   </sheetData>
@@ -545,6 +598,23 @@
             </x14:sparkline>
           </x14:sparklines>
         </x14:sparklineGroup>
+        <x14:sparklineGroup displayEmptyCellsAs="gap" markers="1" dateAxis="1">
+          <x14:colorSeries rgb="FF0000FF"/>
+          <x14:colorNegative rgb="FFFF8000"/>
+          <x14:colorAxis rgb="FFFF00FF"/>
+          <x14:colorMarkers rgb="FFFFC000"/>
+          <x14:colorFirst rgb="FF00A000"/>
+          <x14:colorLast rgb="FFA000A0"/>
+          <x14:colorHigh rgb="FFFF0000"/>
+          <x14:colorLow rgb="FF00A0A0"/>
+          <xm:f>Sheet1!A10:H10</xm:f>
+          <x14:sparklines>
+            <x14:sparkline>
+              <xm:f>Sheet1!A5:H5</xm:f>
+              <xm:sqref>J5</xm:sqref>
+            </x14:sparkline>
+          </x14:sparklines>
+        </x14:sparklineGroup>
       </x14:sparklineGroups>
     </ext>
   </extLst>

</xml_diff>